<commit_message>
Updates files and tables
</commit_message>
<xml_diff>
--- a/Files Data.xlsx
+++ b/Files Data.xlsx
@@ -35444,7 +35444,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="19.57642857142857" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -36555,21 +36555,63 @@
     <row r="53" ht="18.75" customHeight="1">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ختام الذكصولوجيات</t>
+          <t>مارينا الراهبة</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>{01F803BF-F3EE-41F7-A0D0-515D7826AABB}</t>
+          <t>{6700ECA7-ED07-426B-8798-9D373D9CE114}</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>489</v>
       </c>
       <c r="D53" t="n">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="E53" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>الأرشيدياكون حبيب جرجس</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>{8A41060F-BB1F-4290-BD18-2C0336114DEC}</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>497</v>
+      </c>
+      <c r="D54" t="n">
+        <v>502</v>
+      </c>
+      <c r="E54" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ختام الذكصولوجيات</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>{01F803BF-F3EE-41F7-A0D0-515D7826AABB}</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>503</v>
+      </c>
+      <c r="D55" t="n">
+        <v>508</v>
+      </c>
+      <c r="E55" t="n">
         <v>6</v>
       </c>
     </row>
@@ -43512,7 +43554,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="41.005" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -45295,210 +45337,231 @@
     <row r="85" ht="18.75" customHeight="1">
       <c r="A85" t="inlineStr">
         <is>
-          <t>الباب الثالث</t>
+          <t>الملاك رافائيل</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>{E5B98BC1-9C9D-42EC-BB16-E848179FB9DC}</t>
+          <t>{0699D0FB-032D-4E0B-A155-A685C1B680A4}</t>
         </is>
       </c>
       <c r="C85" t="n">
         <v>1977</v>
       </c>
       <c r="D85" t="n">
-        <v>1977</v>
+        <v>1990</v>
       </c>
       <c r="E85" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="86" ht="18.75" customHeight="1">
       <c r="A86" t="inlineStr">
         <is>
-          <t>أعروس الفادي القبطية</t>
+          <t>الباب الثالث</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>{3CBD5E49-3BE4-475A-A6D3-2858A4DB1030}</t>
+          <t>{E5B98BC1-9C9D-42EC-BB16-E848179FB9DC}</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1978</v>
+        <v>1991</v>
       </c>
       <c r="D86" t="n">
-        <v>2006</v>
+        <v>1991</v>
       </c>
       <c r="E86" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87" ht="18.75" customHeight="1">
       <c r="A87" t="inlineStr">
         <is>
-          <t>انظروا يديه تأملوا رجليه</t>
+          <t>أعروس الفادي القبطية</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>{E1A31474-7F00-4B7D-90FD-A67415E32872}</t>
+          <t>{3CBD5E49-3BE4-475A-A6D3-2858A4DB1030}</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2007</v>
+        <v>1992</v>
       </c>
       <c r="D87" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="E87" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
     </row>
     <row r="88" ht="18.75" customHeight="1">
       <c r="A88" t="inlineStr">
         <is>
-          <t>رحلة الصوم الكبير</t>
+          <t>انظروا يديه تأملوا رجليه</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>{11755A37-6BDF-4E72-9537-F39867C5BB7D}</t>
+          <t>{E1A31474-7F00-4B7D-90FD-A67415E32872}</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="D88" t="n">
-        <v>2028</v>
+        <v>2035</v>
       </c>
       <c r="E88" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="89" ht="18.75" customHeight="1">
       <c r="A89" t="inlineStr">
         <is>
-          <t>عند شق الفجر باكر</t>
+          <t>رحلة الصوم الكبير</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>{D4859CD1-25CE-465C-846E-A0311D24DB66}</t>
+          <t>{11755A37-6BDF-4E72-9537-F39867C5BB7D}</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2029</v>
+        <v>2036</v>
       </c>
       <c r="D89" t="n">
-        <v>2055</v>
+        <v>2042</v>
       </c>
       <c r="E89" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
     </row>
     <row r="90" ht="18.75" customHeight="1">
       <c r="A90" t="inlineStr">
         <is>
-          <t>قام حقا</t>
+          <t>عند شق الفجر باكر</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>{4615B620-F94D-4CAD-843A-EB32E8369AAB}</t>
+          <t>{D4859CD1-25CE-465C-846E-A0311D24DB66}</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2056</v>
+        <v>2043</v>
       </c>
       <c r="D90" t="n">
         <v>2069</v>
       </c>
       <c r="E90" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="91" ht="18.75" customHeight="1">
       <c r="A91" t="inlineStr">
         <is>
-          <t>كنيستي أرجو لك</t>
+          <t>قام حقا</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>{8A08F2A7-DAF4-4998-9EF9-8221744F0038}</t>
+          <t>{4615B620-F94D-4CAD-843A-EB32E8369AAB}</t>
         </is>
       </c>
       <c r="C91" t="n">
         <v>2070</v>
       </c>
       <c r="D91" t="n">
-        <v>2080</v>
+        <v>2083</v>
       </c>
       <c r="E91" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="92" ht="18.75" customHeight="1">
       <c r="A92" t="inlineStr">
         <is>
-          <t>كنيستي القبطية كنيسة الإله</t>
+          <t>كنيستي أرجو لك</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>{B1A30565-0CDB-40D5-8B05-21F68D5C9160}</t>
+          <t>{8A08F2A7-DAF4-4998-9EF9-8221744F0038}</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2081</v>
+        <v>2084</v>
       </c>
       <c r="D92" t="n">
-        <v>2107</v>
+        <v>2094</v>
       </c>
       <c r="E92" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
     </row>
     <row r="93" ht="18.75" customHeight="1">
       <c r="A93" t="inlineStr">
         <is>
-          <t>كنيستي القبطية نشرت المسيحية</t>
+          <t>كنيستي القبطية كنيسة الإله</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>{AB60D02D-F80E-4E53-B0A0-3A54593EB31B}</t>
+          <t>{B1A30565-0CDB-40D5-8B05-21F68D5C9160}</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2108</v>
+        <v>2095</v>
       </c>
       <c r="D93" t="n">
-        <v>2120</v>
+        <v>2121</v>
       </c>
       <c r="E93" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
     </row>
     <row r="94" ht="18.75" customHeight="1">
       <c r="A94" t="inlineStr">
         <is>
+          <t>كنيستي القبطية نشرت المسيحية</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>{AB60D02D-F80E-4E53-B0A0-3A54593EB31B}</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>2122</v>
+      </c>
+      <c r="D94" t="n">
+        <v>2134</v>
+      </c>
+      <c r="E94" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
           <t>يا ربنا مولى السلام</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>{325B4DE6-FA63-4B6D-827F-BCC78EF1FEC9}</t>
         </is>
       </c>
-      <c r="C94" t="n">
-        <v>2121</v>
-      </c>
-      <c r="D94" t="n">
-        <v>2164</v>
-      </c>
-      <c r="E94" t="n">
+      <c r="C95" t="n">
+        <v>2135</v>
+      </c>
+      <c r="D95" t="n">
+        <v>2178</v>
+      </c>
+      <c r="E95" t="n">
         <v>44</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: saints calendar base - hide and show
</commit_message>
<xml_diff>
--- a/Files Data.xlsx
+++ b/Files Data.xlsx
@@ -35444,7 +35444,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="19.57642857142857" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -36555,21 +36555,63 @@
     <row r="53" ht="18.75" customHeight="1">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ختام الذكصولوجيات</t>
+          <t>مارينا الراهبة</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>{01F803BF-F3EE-41F7-A0D0-515D7826AABB}</t>
+          <t>{6700ECA7-ED07-426B-8798-9D373D9CE114}</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>489</v>
       </c>
       <c r="D53" t="n">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="E53" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>الأرشيدياكون حبيب جرجس</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>{8A41060F-BB1F-4290-BD18-2C0336114DEC}</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>497</v>
+      </c>
+      <c r="D54" t="n">
+        <v>502</v>
+      </c>
+      <c r="E54" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ختام الذكصولوجيات</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>{01F803BF-F3EE-41F7-A0D0-515D7826AABB}</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>503</v>
+      </c>
+      <c r="D55" t="n">
+        <v>508</v>
+      </c>
+      <c r="E55" t="n">
         <v>6</v>
       </c>
     </row>
@@ -43512,7 +43554,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="41.005" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -45295,210 +45337,231 @@
     <row r="85" ht="18.75" customHeight="1">
       <c r="A85" t="inlineStr">
         <is>
-          <t>الباب الثالث</t>
+          <t>الملاك رافائيل</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>{E5B98BC1-9C9D-42EC-BB16-E848179FB9DC}</t>
+          <t>{0699D0FB-032D-4E0B-A155-A685C1B680A4}</t>
         </is>
       </c>
       <c r="C85" t="n">
         <v>1977</v>
       </c>
       <c r="D85" t="n">
-        <v>1977</v>
+        <v>1990</v>
       </c>
       <c r="E85" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
     </row>
     <row r="86" ht="18.75" customHeight="1">
       <c r="A86" t="inlineStr">
         <is>
-          <t>أعروس الفادي القبطية</t>
+          <t>الباب الثالث</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>{3CBD5E49-3BE4-475A-A6D3-2858A4DB1030}</t>
+          <t>{E5B98BC1-9C9D-42EC-BB16-E848179FB9DC}</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1978</v>
+        <v>1991</v>
       </c>
       <c r="D86" t="n">
-        <v>2006</v>
+        <v>1991</v>
       </c>
       <c r="E86" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87" ht="18.75" customHeight="1">
       <c r="A87" t="inlineStr">
         <is>
-          <t>انظروا يديه تأملوا رجليه</t>
+          <t>أعروس الفادي القبطية</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>{E1A31474-7F00-4B7D-90FD-A67415E32872}</t>
+          <t>{3CBD5E49-3BE4-475A-A6D3-2858A4DB1030}</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2007</v>
+        <v>1992</v>
       </c>
       <c r="D87" t="n">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="E87" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
     </row>
     <row r="88" ht="18.75" customHeight="1">
       <c r="A88" t="inlineStr">
         <is>
-          <t>رحلة الصوم الكبير</t>
+          <t>انظروا يديه تأملوا رجليه</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>{11755A37-6BDF-4E72-9537-F39867C5BB7D}</t>
+          <t>{E1A31474-7F00-4B7D-90FD-A67415E32872}</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="D88" t="n">
-        <v>2028</v>
+        <v>2035</v>
       </c>
       <c r="E88" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="89" ht="18.75" customHeight="1">
       <c r="A89" t="inlineStr">
         <is>
-          <t>عند شق الفجر باكر</t>
+          <t>رحلة الصوم الكبير</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>{D4859CD1-25CE-465C-846E-A0311D24DB66}</t>
+          <t>{11755A37-6BDF-4E72-9537-F39867C5BB7D}</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2029</v>
+        <v>2036</v>
       </c>
       <c r="D89" t="n">
-        <v>2055</v>
+        <v>2042</v>
       </c>
       <c r="E89" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
     </row>
     <row r="90" ht="18.75" customHeight="1">
       <c r="A90" t="inlineStr">
         <is>
-          <t>قام حقا</t>
+          <t>عند شق الفجر باكر</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>{4615B620-F94D-4CAD-843A-EB32E8369AAB}</t>
+          <t>{D4859CD1-25CE-465C-846E-A0311D24DB66}</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2056</v>
+        <v>2043</v>
       </c>
       <c r="D90" t="n">
         <v>2069</v>
       </c>
       <c r="E90" t="n">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="91" ht="18.75" customHeight="1">
       <c r="A91" t="inlineStr">
         <is>
-          <t>كنيستي أرجو لك</t>
+          <t>قام حقا</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>{8A08F2A7-DAF4-4998-9EF9-8221744F0038}</t>
+          <t>{4615B620-F94D-4CAD-843A-EB32E8369AAB}</t>
         </is>
       </c>
       <c r="C91" t="n">
         <v>2070</v>
       </c>
       <c r="D91" t="n">
-        <v>2080</v>
+        <v>2083</v>
       </c>
       <c r="E91" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="92" ht="18.75" customHeight="1">
       <c r="A92" t="inlineStr">
         <is>
-          <t>كنيستي القبطية كنيسة الإله</t>
+          <t>كنيستي أرجو لك</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>{B1A30565-0CDB-40D5-8B05-21F68D5C9160}</t>
+          <t>{8A08F2A7-DAF4-4998-9EF9-8221744F0038}</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2081</v>
+        <v>2084</v>
       </c>
       <c r="D92" t="n">
-        <v>2107</v>
+        <v>2094</v>
       </c>
       <c r="E92" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
     </row>
     <row r="93" ht="18.75" customHeight="1">
       <c r="A93" t="inlineStr">
         <is>
-          <t>كنيستي القبطية نشرت المسيحية</t>
+          <t>كنيستي القبطية كنيسة الإله</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>{AB60D02D-F80E-4E53-B0A0-3A54593EB31B}</t>
+          <t>{B1A30565-0CDB-40D5-8B05-21F68D5C9160}</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2108</v>
+        <v>2095</v>
       </c>
       <c r="D93" t="n">
-        <v>2120</v>
+        <v>2121</v>
       </c>
       <c r="E93" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
     </row>
     <row r="94" ht="18.75" customHeight="1">
       <c r="A94" t="inlineStr">
         <is>
+          <t>كنيستي القبطية نشرت المسيحية</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>{AB60D02D-F80E-4E53-B0A0-3A54593EB31B}</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>2122</v>
+      </c>
+      <c r="D94" t="n">
+        <v>2134</v>
+      </c>
+      <c r="E94" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
           <t>يا ربنا مولى السلام</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>{325B4DE6-FA63-4B6D-827F-BCC78EF1FEC9}</t>
         </is>
       </c>
-      <c r="C94" t="n">
-        <v>2121</v>
-      </c>
-      <c r="D94" t="n">
-        <v>2164</v>
-      </c>
-      <c r="E94" t="n">
+      <c r="C95" t="n">
+        <v>2135</v>
+      </c>
+      <c r="D95" t="n">
+        <v>2178</v>
+      </c>
+      <c r="E95" t="n">
         <v>44</v>
       </c>
     </row>

</xml_diff>